<commit_message>
v2 report: keep row order matching v1 (no longer sorted by rank)
</commit_message>
<xml_diff>
--- a/G2_Coding_Challenge_Review_Results_v2.xlsx
+++ b/G2_Coding_Challenge_Review_Results_v2.xlsx
@@ -60,8 +60,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -72,8 +72,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -604,16 +604,16 @@
     </row>
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>127156040_ASHLEY</t>
+          <t>127156011_ASHLEY</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Q27</t>
+          <t>Q15</t>
         </is>
       </c>
       <c r="D2" s="4" t="n">
@@ -626,13 +626,13 @@
         <v>15</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>15</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -646,12 +646,12 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Correct BFS tree reconstruction and level-sum aggregation; Handles empty tree, single node, negatives, mixed nulls</t>
+          <t>Matches Example 1 (3x4-&gt;65) and correctly handles the 1x1 mandatory edge case (42-&gt;42); Elegant single border-sum condition (i==0 or i==r-1 or j==0 or j==c-1) avoids double counting corners; Code-inspection confirms the condition also correctly handles single-row/single-column matrices even though untested</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>None noted</t>
+          <t>Mandatory edge case 'single row or single column' was never exercised in the submitted test evidence (Output.png) - the third run (3x5) is just another normal-size matrix, not an edge case; No automated/assert-based tests, only manual terminal runs; No input validation or comments</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
@@ -667,16 +667,16 @@
     </row>
     <row r="3" ht="70" customHeight="1">
       <c r="A3" s="2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>127156067_ASHLEY</t>
+          <t>127156017_ASHLEY</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Q07</t>
+          <t>Q29</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
@@ -689,13 +689,13 @@
         <v>15</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
@@ -709,12 +709,12 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Perfect stack-based bracket matching; Correctly reports first error index for all error types</t>
+          <t>Correct two-pointer sweep with proper tie handling (&lt; not &lt;=); O(n log n) optimal</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>None noted</t>
+          <t>Add input validation; Add comments; No explicit test cases included</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
@@ -724,22 +724,22 @@
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
+          <t>Strong submission with correct logic and only minor polish gaps.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="70" customHeight="1">
       <c r="A4" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>127156116_ASHLEY</t>
+          <t>127156026_ASHLEY</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Q05</t>
+          <t>Q01</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
@@ -752,13 +752,13 @@
         <v>15</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -772,12 +772,12 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>All 6 rules correctly implemented in correct order; Handles empty input, multiple failures, embedded spaces correctly</t>
+          <t>Correct regex tokenization and Counter usage; Correct dual-key sort (freq desc, alpha asc)</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>None noted</t>
+          <t>Missing docstring; No explicit error handling</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr">
@@ -793,35 +793,35 @@
     </row>
     <row r="5" ht="70" customHeight="1">
       <c r="A5" s="2" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>127156074_ASHLEY</t>
+          <t>127156027_ASHLEY</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Q14</t>
+          <t>Q19</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>10</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
@@ -835,60 +835,60 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Correct median-of-halves quartile method for even/odd arrays; Correct IQR bounds and order-preserving output</t>
+          <t>Correct composite comparator (dept asc, score desc, name asc); Handles decimal scores and format preservation</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>Input prompts are verbose, not matching typical stdin convention</t>
+          <t>No input validation; No test file provided</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Missing test coverage</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
+          <t>Strong submission with correct logic and only minor polish gaps.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="70" customHeight="1">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>127156039_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Q22</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>127156150_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Q02</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="I6" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -898,37 +898,37 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Correct single-pass top-2 distinct tracking; Handles duplicates, negatives, all-equal values correctly</t>
+          <t>Correct email validation logic (id required, exactly one '@', non-empty local/domain parts) and correct duplicate-tracking design using dict keyed by id; Design intent is correct: last-write-wins per id, matching the expected 'valid/rejected/duplicates_removed' metrics</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Add inline comments explaining tracking logic</t>
+          <t>CRITICAL: extracted source is non-runnable as submitted - confirmed via execution, raises 'IndentationError: unexpected indent' on the 'record=records[id]' line because it sits outside the for-loop (the preceding 'duplicates_removed=...' line is unindented, closing the loop early) while the print statements below it are still indented as if inside the loop; The single stdin/stdout transcript captured in the notebook could not have been produced by this exact code given the IndentationError, indicating the recorded output does not match the submitted source; No automated tests, only one manual run</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CRITICAL: Non-runnable submission (IndentationError); Test evidence mismatch with submitted code</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
+          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: Non-runnable submission (IndentationError).</t>
         </is>
       </c>
     </row>
     <row r="7" ht="70" customHeight="1">
       <c r="A7" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>127156062_ASHLEY</t>
+          <t>127156040_ASHLEY</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Q04</t>
+          <t>Q27</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
@@ -944,10 +944,10 @@
         <v>15</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -961,12 +961,12 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Correct grouping/averaging and multi-key sort; Tested decimal scores, tied averages, single-record depts</t>
+          <t>Correct BFS tree reconstruction and level-sum aggregation; Handles empty tree, single node, negatives, mixed nulls</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t>Variable names could be more descriptive; No input validation</t>
+          <t>None noted</t>
         </is>
       </c>
       <c r="N7" s="3" t="inlineStr">
@@ -982,16 +982,16 @@
     </row>
     <row r="8" ht="70" customHeight="1">
       <c r="A8" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>127156026_ASHLEY</t>
+          <t>127156062_ASHLEY</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Q01</t>
+          <t>Q04</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
@@ -1004,13 +1004,13 @@
         <v>15</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>13</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -1024,12 +1024,12 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Correct regex tokenization and Counter usage; Correct dual-key sort (freq desc, alpha asc)</t>
+          <t>Correct grouping/averaging and multi-key sort; Tested decimal scores, tied averages, single-record depts</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Missing docstring; No explicit error handling</t>
+          <t>Variable names could be more descriptive; No input validation</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
@@ -1044,40 +1044,40 @@
       </c>
     </row>
     <row r="9" ht="70" customHeight="1">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
+      <c r="A9" s="5" t="n">
+        <v>25</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>127156113_Ashley</t>
+          <t>127179036_ASHLEY</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Q20</t>
+          <t>Q04</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>96</v>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
+        <v>6</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1087,104 +1087,104 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Correct unbounded coin-change DP with sentinel for impossibility; Both examples pass</t>
+          <t>Correct grouping and averaging math</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>No explicit target=0 test; No comments explaining DP approach</t>
+          <t>CRITICAL: sorts alphabetically instead of by average desc then name asc; Uses string comparison for max instead of numeric; No testing against Example 2 which reveals the bug</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>FAIL_EXAMPLE_2; WRONG_SORT_ORDER</t>
         </is>
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
+          <t>Weak/failing submission with critical correctness issues.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="70" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
+      <c r="A10" s="5" t="n">
+        <v>28</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>127179065_ASHLEY</t>
+          <t>127156063_ASHLEY</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Q06</t>
+          <t>Q09</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>96</v>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
+        <v>2</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Correct monotonic-deque sliding window, O(n) complexity; Handles k=1, k=n, negatives, decimals correctly</t>
+          <t>Code is syntactically clean</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>Poor variable naming (mbers, dec_deque, inptokens); Missing comments explaining deque logic</t>
+          <t>CRITICAL: Wrong problem solved (Q10 code submitted instead of Q09); No earliest-second-occurrence logic present</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CRITICAL: Wrong problem solved</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>Excellent, near-flawless submission. Strong hire signal for this challenge. Possible AI assistance signals noted (informational only, not penalized).</t>
+          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: Wrong problem solved.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="70" customHeight="1">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
+      <c r="A11" s="6" t="n">
+        <v>19</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>127156011_ASHLEY</t>
+          <t>127156063_ASHLEY</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Q15</t>
+          <t>Q10</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>10</v>
@@ -1193,17 +1193,17 @@
         <v>15</v>
       </c>
       <c r="G11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="H11" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="I11" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="I11" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1213,37 +1213,37 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>Matches Example 1 (3x4-&gt;65) and correctly handles the 1x1 mandatory edge case (42-&gt;42); Elegant single border-sum condition (i==0 or i==r-1 or j==0 or j==c-1) avoids double counting corners; Code-inspection confirms the condition also correctly handles single-row/single-column matrices even though untested</t>
+          <t>Correct grouping/counting/sorting logic; Correct problem interpretation</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>Mandatory edge case 'single row or single column' was never exercised in the submitted test evidence (Output.png) - the third run (3x5) is just another normal-size matrix, not an edge case; No automated/assert-based tests, only manual terminal runs; No input validation or comments</t>
+          <t>CRITICAL: whitespace not stripped from input, causing wrong event names in output (demonstrated failure in own test); No input validation; Minimal testing</t>
         </is>
       </c>
       <c r="N11" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CRITICAL_BUG: whitespace handling</t>
         </is>
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
+          <t>Partial solution with a significant functional or logic bug; needs follow-up. Critical concern(s): CRITICAL_BUG: whitespace handling.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="70" customHeight="1">
       <c r="A12" s="2" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>127156017_ASHLEY</t>
+          <t>127156067_ASHLEY</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Q29</t>
+          <t>Q07</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
@@ -1256,13 +1256,13 @@
         <v>15</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -1276,12 +1276,12 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>Correct two-pointer sweep with proper tie handling (&lt; not &lt;=); O(n log n) optimal</t>
+          <t>Perfect stack-based bracket matching; Correctly reports first error index for all error types</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Add input validation; Add comments; No explicit test cases included</t>
+          <t>None noted</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
@@ -1291,45 +1291,45 @@
       </c>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Strong submission with correct logic and only minor polish gaps.</t>
+          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="70" customHeight="1">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
+      <c r="A13" s="5" t="n">
+        <v>27</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>127156082_ASHLEY</t>
+          <t>127156072_ASHLEY</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Q17</t>
+          <t>Q24</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
+        <v>2</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1339,37 +1339,37 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>Correct BFS shortest path implementation; Handles disconnected graphs and duplicate edges correctly</t>
+          <t>Reads input format correctly</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>No explicit test for source==destination; No comments explaining algorithm</t>
+          <t>CRITICAL: counts node degree instead of connected components; No DFS/BFS/Union-Find implemented; Second attempt has runtime errors; Uses interactive input instead of standard format</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CRITICAL: Algorithm completely wrong; Runtime errors present</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Strong submission with correct logic and only minor polish gaps.</t>
+          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: Algorithm completely wrong.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="70" customHeight="1">
       <c r="A14" s="2" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>127156105_ASHLEY</t>
+          <t>127156074_ASHLEY</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Q11</t>
+          <t>Q14</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
@@ -1382,13 +1382,13 @@
         <v>15</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -1402,12 +1402,12 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>Correct hashmap tie-break logic (smallest j then smallest i); All provided test cases pass</t>
+          <t>Correct median-of-halves quartile method for even/odd arrays; Correct IQR bounds and order-preserving output</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>No comments explaining tie-break strategy; Limited edge case testing (duplicates, negatives)</t>
+          <t>Input prompts are verbose, not matching typical stdin convention</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
@@ -1417,41 +1417,41 @@
       </c>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Strong submission with correct logic and only minor polish gaps.</t>
+          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="70" customHeight="1">
       <c r="A15" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>127156027_ASHLEY</t>
+          <t>127156082_ASHLEY</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Q19</t>
+          <t>Q17</t>
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>10</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H15" s="4" t="n">
         <v>13</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
@@ -1465,17 +1465,17 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>Correct composite comparator (dept asc, score desc, name asc); Handles decimal scores and format preservation</t>
+          <t>Correct BFS shortest path implementation; Handles disconnected graphs and duplicate edges correctly</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>No input validation; No test file provided</t>
+          <t>No explicit test for source==destination; No comments explaining algorithm</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
         <is>
-          <t>Missing test coverage</t>
+          <t>None</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr">
@@ -1548,210 +1548,210 @@
       </c>
     </row>
     <row r="17" ht="70" customHeight="1">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
+      <c r="A17" s="6" t="n">
+        <v>20</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>127179051_ASHLEY</t>
+          <t>127156100_ASHLEY</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Q13</t>
+          <t>Q28</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F17" s="4" t="n">
         <v>14</v>
       </c>
       <c r="G17" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="H17" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="I17" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="I17" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>Correct sliding-window algorithm structure; Correct tie-break to earliest start index</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: uses ch.lower() breaking case-sensitivity requirement, causing wrong results on mixed-case input (e.g. 'AaA'); No case-sensitivity test cases</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL_BUG: case-sensitivity violation</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Partial solution with a significant functional or logic bug; needs follow-up. Critical concern(s): CRITICAL_BUG: case-sensitivity violation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>127156103_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Q26</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Correct AND-filter logic and operator dispatch; Maintains original record order and formatting</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: prints debug header '*****OUTPUT*****' violating output spec; No error handling for malformed input</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: Output format violation (debug header)</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>Solid attempt with correct core logic but noticeable gaps in testing/quality. Critical concern(s): CRITICAL: Output format violation (debug header).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="70" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>127156105_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="I19" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
-        <is>
-          <t>Correct recursive flattening, arrays preserved, lexicographic sort; Handles null values and empty objects correctly</t>
-        </is>
-      </c>
-      <c r="M17" s="3" t="inlineStr">
-        <is>
-          <t>Off-by-one bug in depth limit check (allows 21 levels instead of 20); No test file provided</t>
-        </is>
-      </c>
-      <c r="N17" s="3" t="inlineStr">
-        <is>
-          <t>depth_limit_bug</t>
-        </is>
-      </c>
-      <c r="O17" s="3" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Correct hashmap tie-break logic (smallest j then smallest i); All provided test cases pass</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>No comments explaining tie-break strategy; Limited edge case testing (duplicates, negatives)</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O19" s="3" t="inlineStr">
         <is>
           <t>Strong submission with correct logic and only minor polish gaps.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="70" customHeight="1">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>127156021_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Q23</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="n">
+    <row r="20" ht="70" customHeight="1">
+      <c r="A20" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>127156113_Ashley</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Q20</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
         <v>45</v>
-      </c>
-      <c r="E18" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G18" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="H18" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="I18" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="L18" s="3" t="inlineStr">
-        <is>
-          <t>Correct O(n) set-based sequence-start detection matching AI focus guidance; Both provided examples pass (length 4, length 5) plus an additional manual test with duplicates</t>
-        </is>
-      </c>
-      <c r="M18" s="3" t="inlineStr">
-        <is>
-          <t>No negative-number test recorded despite being a stated edge case; No comments or error handling; File is misleadingly named 'Longest_common_subsequence.py' though it correctly solves Longest Consecutive Sequence; Contains an extra OUTPUT.md file documenting manual test runs, alongside the problem-statement markdown</t>
-        </is>
-      </c>
-      <c r="N18" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="O18" s="3" t="inlineStr">
-        <is>
-          <t>Strong submission with correct logic and only minor polish gaps. Possible AI assistance signals noted (informational only, not penalized).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="70" customHeight="1">
-      <c r="A19" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>127156103_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Q26</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>32</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="H19" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>75</v>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L19" s="3" t="inlineStr">
-        <is>
-          <t>Correct AND-filter logic and operator dispatch; Maintains original record order and formatting</t>
-        </is>
-      </c>
-      <c r="M19" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: prints debug header '*****OUTPUT*****' violating output spec; No error handling for malformed input</t>
-        </is>
-      </c>
-      <c r="N19" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: Output format violation (debug header)</t>
-        </is>
-      </c>
-      <c r="O19" s="3" t="inlineStr">
-        <is>
-          <t>Solid attempt with correct core logic but noticeable gaps in testing/quality. Critical concern(s): CRITICAL: Output format violation (debug header).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="70" customHeight="1">
-      <c r="A20" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>127156063_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Q10</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>20</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>10</v>
@@ -1760,609 +1760,609 @@
         <v>15</v>
       </c>
       <c r="G20" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>Correct unbounded coin-change DP with sentinel for impossibility; Both examples pass</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>No explicit target=0 test; No comments explaining DP approach</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="70" customHeight="1">
+      <c r="A21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>127156116_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Q05</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E21" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="I20" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="F21" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
-        <is>
-          <t>Correct grouping/counting/sorting logic; Correct problem interpretation</t>
-        </is>
-      </c>
-      <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: whitespace not stripped from input, causing wrong event names in output (demonstrated failure in own test); No input validation; Minimal testing</t>
-        </is>
-      </c>
-      <c r="N20" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL_BUG: whitespace handling</t>
-        </is>
-      </c>
-      <c r="O20" s="3" t="inlineStr">
-        <is>
-          <t>Partial solution with a significant functional or logic bug; needs follow-up. Critical concern(s): CRITICAL_BUG: whitespace handling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="70" customHeight="1">
-      <c r="A21" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>127156100_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Q28</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E21" s="4" t="n">
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>All 6 rules correctly implemented in correct order; Handles empty input, multiple failures, embedded spaces correctly</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>None noted</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
+      <c r="A22" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>127156149_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Q25</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Attempted a cache structure using dictionary</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: no LRU eviction mechanism, no doubly-linked list, wrong input format (interactive instead of command parsing); Undefined variable causes runtime crash; Does not match provided examples</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: No LRU logic implemented; CRITICAL: Runtime crash bug</t>
+        </is>
+      </c>
+      <c r="O22" s="3" t="inlineStr">
+        <is>
+          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: No LRU logic implemented; CRITICAL: Runtime crash bug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="70" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>127156150_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Q02</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="H23" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="I23" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Correct single-pass top-2 distinct tracking; Handles duplicates, negatives, all-equal values correctly</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Add inline comments explaining tracking logic</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O23" s="3" t="inlineStr">
+        <is>
+          <t>Excellent, near-flawless submission. Strong hire signal for this challenge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="70" customHeight="1">
+      <c r="A24" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>127179051_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Correct recursive flattening, arrays preserved, lexicographic sort; Handles null values and empty objects correctly</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>Off-by-one bug in depth limit check (allows 21 levels instead of 20); No test file provided</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>depth_limit_bug</t>
+        </is>
+      </c>
+      <c r="O24" s="3" t="inlineStr">
+        <is>
+          <t>Strong submission with correct logic and only minor polish gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="70" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>127179056_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Q08</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H25" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="I25" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Correct percentage calculation and output format for complete rows</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: operator precedence bug causes IndexError on short rows (Example 2 fails); Code hardcodes input instead of reading from stdin</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>RUNTIME_ERROR on short rows; LOGIC_ERROR: operator precedence</t>
+        </is>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t>Weak/failing submission with critical correctness issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="70" customHeight="1">
+      <c r="A26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>127179065_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Q06</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G26" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="G21" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H21" s="4" t="n">
+      <c r="H26" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="I21" s="6" t="n">
-        <v>55</v>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L21" s="3" t="inlineStr">
-        <is>
-          <t>Correct sliding-window algorithm structure; Correct tie-break to earliest start index</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: uses ch.lower() breaking case-sensitivity requirement, causing wrong results on mixed-case input (e.g. 'AaA'); No case-sensitivity test cases</t>
-        </is>
-      </c>
-      <c r="N21" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL_BUG: case-sensitivity violation</t>
-        </is>
-      </c>
-      <c r="O21" s="3" t="inlineStr">
-        <is>
-          <t>Partial solution with a significant functional or logic bug; needs follow-up. Critical concern(s): CRITICAL_BUG: case-sensitivity violation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="70" customHeight="1">
-      <c r="A22" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>127179056_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Q08</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E22" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G22" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I22" s="7" t="n">
-        <v>41</v>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L22" s="3" t="inlineStr">
-        <is>
-          <t>Correct percentage calculation and output format for complete rows</t>
-        </is>
-      </c>
-      <c r="M22" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: operator precedence bug causes IndexError on short rows (Example 2 fails); Code hardcodes input instead of reading from stdin</t>
-        </is>
-      </c>
-      <c r="N22" s="3" t="inlineStr">
-        <is>
-          <t>RUNTIME_ERROR on short rows; LOGIC_ERROR: operator precedence</t>
-        </is>
-      </c>
-      <c r="O22" s="3" t="inlineStr">
-        <is>
-          <t>Weak/failing submission with critical correctness issues.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="70" customHeight="1">
-      <c r="A23" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>127156039_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Q22</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="G23" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="H23" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I23" s="7" t="n">
-        <v>37</v>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L23" s="3" t="inlineStr">
-        <is>
-          <t>Correct email validation logic (id required, exactly one '@', non-empty local/domain parts) and correct duplicate-tracking design using dict keyed by id; Design intent is correct: last-write-wins per id, matching the expected 'valid/rejected/duplicates_removed' metrics</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: extracted source is non-runnable as submitted - confirmed via execution, raises 'IndentationError: unexpected indent' on the 'record=records[id]' line because it sits outside the for-loop (the preceding 'duplicates_removed=...' line is unindented, closing the loop early) while the print statements below it are still indented as if inside the loop; The single stdin/stdout transcript captured in the notebook could not have been produced by this exact code given the IndentationError, indicating the recorded output does not match the submitted source; No automated tests, only one manual run</t>
-        </is>
-      </c>
-      <c r="N23" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: Non-runnable submission (IndentationError); Test evidence mismatch with submitted code</t>
-        </is>
-      </c>
-      <c r="O23" s="3" t="inlineStr">
-        <is>
-          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: Non-runnable submission (IndentationError).</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="70" customHeight="1">
-      <c r="A24" s="7" t="n">
+      <c r="I26" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Correct monotonic-deque sliding window, O(n) complexity; Handles k=1, k=n, negatives, decimals correctly</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>Poor variable naming (mbers, dec_deque, inptokens); Missing comments explaining deque logic</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>Excellent, near-flawless submission. Strong hire signal for this challenge. Possible AI assistance signals noted (informational only, not penalized).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="70" customHeight="1">
+      <c r="A27" s="5" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>127179066_ASHLEY</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Q03</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F24" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="G24" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H24" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I24" s="7" t="n">
-        <v>36</v>
-      </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>Correct dedup logic and score validation design inside function</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: function defined but never called - produces no output; Tie-break bug uses &gt; instead of &gt;= for equal timestamps; No test cases included</t>
-        </is>
-      </c>
-      <c r="N24" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: No program output produced</t>
-        </is>
-      </c>
-      <c r="O24" s="3" t="inlineStr">
-        <is>
-          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: No program output produced.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="70" customHeight="1">
-      <c r="A25" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>127179060_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Q09</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G25" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I25" s="7" t="n">
-        <v>36</v>
-      </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L25" s="3" t="inlineStr">
-        <is>
-          <t>Correct hashmap-based first-seen-index design with early exit on second occurrence, matching the expected algorithm</t>
-        </is>
-      </c>
-      <c r="M25" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: code uses '//' (C/Java-style) instead of '#' for comments on lines 1 and 3, causing a Python SyntaxError - the submitted file does not run as-is; results.txt transcript shows input prompts ('enter no of elements') that do not exist anywhere in the submitted code, indicating the recorded test evidence does not correspond to the actual submitted file; No error handling or input validation</t>
-        </is>
-      </c>
-      <c r="N25" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: Non-runnable submission (SyntaxError from // comments); Test evidence mismatch with submitted code</t>
-        </is>
-      </c>
-      <c r="O25" s="3" t="inlineStr">
-        <is>
-          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: Non-runnable submission (SyntaxError from // comments).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="70" customHeight="1">
-      <c r="A26" s="7" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>127179036_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Q04</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F26" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I26" s="7" t="n">
-        <v>35</v>
-      </c>
-      <c r="J26" s="7" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L26" s="3" t="inlineStr">
-        <is>
-          <t>Correct grouping and averaging math</t>
-        </is>
-      </c>
-      <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: sorts alphabetically instead of by average desc then name asc; Uses string comparison for max instead of numeric; No testing against Example 2 which reveals the bug</t>
-        </is>
-      </c>
-      <c r="N26" s="3" t="inlineStr">
-        <is>
-          <t>FAIL_EXAMPLE_2; WRONG_SORT_ORDER</t>
-        </is>
-      </c>
-      <c r="O26" s="3" t="inlineStr">
-        <is>
-          <t>Weak/failing submission with critical correctness issues.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="70" customHeight="1">
-      <c r="A27" s="7" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>127156149_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>Q25</t>
         </is>
       </c>
       <c r="D27" s="4" t="n">
         <v>5</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H27" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Correct dedup logic and score validation design inside function</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: function defined but never called - produces no output; Tie-break bug uses &gt; instead of &gt;= for equal timestamps; No test cases included</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>CRITICAL: No program output produced</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: No program output produced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="70" customHeight="1">
+      <c r="A28" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>127156021_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Q23</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Correct O(n) set-based sequence-start detection matching AI focus guidance; Both provided examples pass (length 4, length 5) plus an additional manual test with duplicates</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>No negative-number test recorded despite being a stated edge case; No comments or error handling; File is misleadingly named 'Longest_common_subsequence.py' though it correctly solves Longest Consecutive Sequence; Contains an extra OUTPUT.md file documenting manual test runs, alongside the problem-statement markdown</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O28" s="3" t="inlineStr">
+        <is>
+          <t>Strong submission with correct logic and only minor polish gaps. Possible AI assistance signals noted (informational only, not penalized).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="A29" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>127179060_ASHLEY</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Q09</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G29" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="I27" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="H29" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="K29" s="4" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="L27" s="3" t="inlineStr">
-        <is>
-          <t>Attempted a cache structure using dictionary</t>
-        </is>
-      </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: no LRU eviction mechanism, no doubly-linked list, wrong input format (interactive instead of command parsing); Undefined variable causes runtime crash; Does not match provided examples</t>
-        </is>
-      </c>
-      <c r="N27" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: No LRU logic implemented; CRITICAL: Runtime crash bug</t>
-        </is>
-      </c>
-      <c r="O27" s="3" t="inlineStr">
-        <is>
-          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: No LRU logic implemented; CRITICAL: Runtime crash bug.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="70" customHeight="1">
-      <c r="A28" s="7" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>127156072_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Q24</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I28" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="J28" s="7" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L28" s="3" t="inlineStr">
-        <is>
-          <t>Reads input format correctly</t>
-        </is>
-      </c>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: counts node degree instead of connected components; No DFS/BFS/Union-Find implemented; Second attempt has runtime errors; Uses interactive input instead of standard format</t>
-        </is>
-      </c>
-      <c r="N28" s="3" t="inlineStr">
-        <is>
-          <t>CRITICAL: Algorithm completely wrong; Runtime errors present</t>
-        </is>
-      </c>
-      <c r="O28" s="3" t="inlineStr">
-        <is>
-          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: Algorithm completely wrong.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="70" customHeight="1">
-      <c r="A29" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>127156063_ASHLEY</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Q09</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I29" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>Code is syntactically clean</t>
+          <t>Correct hashmap-based first-seen-index design with early exit on second occurrence, matching the expected algorithm</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>CRITICAL: Wrong problem solved (Q10 code submitted instead of Q09); No earliest-second-occurrence logic present</t>
+          <t>CRITICAL: code uses '//' (C/Java-style) instead of '#' for comments on lines 1 and 3, causing a Python SyntaxError - the submitted file does not run as-is; results.txt transcript shows input prompts ('enter no of elements') that do not exist anywhere in the submitted code, indicating the recorded test evidence does not correspond to the actual submitted file; No error handling or input validation</t>
         </is>
       </c>
       <c r="N29" s="3" t="inlineStr">
         <is>
-          <t>CRITICAL: Wrong problem solved</t>
+          <t>CRITICAL: Non-runnable submission (SyntaxError from // comments); Test evidence mismatch with submitted code</t>
         </is>
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: Wrong problem solved.</t>
+          <t>Weak/failing submission with critical correctness issues. Critical concern(s): CRITICAL: Non-runnable submission (SyntaxError from // comments).</t>
         </is>
       </c>
     </row>

</xml_diff>